<commit_message>
enhance close modal scan qr
</commit_message>
<xml_diff>
--- a/test-data/smoke_test.xlsx
+++ b/test-data/smoke_test.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="36">
   <si>
     <t>scenario</t>
   </si>
@@ -576,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.42578125" style="16" customWidth="1"/>
@@ -621,28 +621,180 @@
     </row>
     <row r="2" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+    </row>
+    <row r="3" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+    </row>
+    <row r="4" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="12"/>
+    </row>
+    <row r="5" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="12"/>
+    </row>
+    <row r="6" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="13" t="s">
+      <c r="B6" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E6" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G6" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12" t="s">
+      <c r="H6" s="12"/>
+      <c r="I6" s="12" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I7" s="12"/>
+    </row>
+    <row r="8" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12" t="s">
         <v>18</v>
       </c>
     </row>
@@ -650,9 +802,21 @@
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" display="testing.b2c.001@gmail.com"/>
     <hyperlink ref="F2" r:id="rId2"/>
+    <hyperlink ref="E4" r:id="rId3" display="testing.b2c.001@gmail.com"/>
+    <hyperlink ref="F4" r:id="rId4"/>
+    <hyperlink ref="E3" r:id="rId5" display="testing.b2c.001@gmail.com"/>
+    <hyperlink ref="F3" r:id="rId6"/>
+    <hyperlink ref="E5" r:id="rId7" display="testing.b2c.001@gmail.com"/>
+    <hyperlink ref="F5" r:id="rId8"/>
+    <hyperlink ref="E6" r:id="rId9" display="testing.b2c.001@gmail.com"/>
+    <hyperlink ref="F6" r:id="rId10"/>
+    <hyperlink ref="E8" r:id="rId11" display="testing.b2c.001@gmail.com"/>
+    <hyperlink ref="F8" r:id="rId12"/>
+    <hyperlink ref="E7" r:id="rId13" display="testing.b2c.001@gmail.com"/>
+    <hyperlink ref="F7" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
 

</xml_diff>